<commit_message>
updated projection code for risk table
</commit_message>
<xml_diff>
--- a/assessment/risk_tables/sc12-jm10_2024.xlsx
+++ b/assessment/risk_tables/sc12-jm10_2024.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leeqi/Library/CloudStorage/GoogleDrive-leeqi@uw.edu/My Drive/SPRFMO/jjm/assessment/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leeqi/Library/CloudStorage/GoogleDrive-leeqi@uw.edu/My Drive/SPRFMO/jjm/assessment/risk_tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{930BE6DF-A360-F042-B0E4-8D0177C5255D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5B1A17A-6C81-7D44-9C32-57AE180D1A99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15120" yWindow="760" windowWidth="15120" windowHeight="18880" xr2:uid="{1354E36E-017E-074A-9785-0738E9F904BC}"/>
+    <workbookView xWindow="38400" yWindow="-8320" windowWidth="14400" windowHeight="25340" xr2:uid="{1354E36E-017E-074A-9785-0738E9F904BC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -637,58 +637,58 @@
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="1">
-        <v>17331</v>
-      </c>
-      <c r="C6" s="1">
-        <v>100</v>
-      </c>
-      <c r="D6" s="1">
-        <v>13489</v>
-      </c>
-      <c r="E6" s="1">
-        <v>94</v>
-      </c>
-      <c r="F6" s="1">
-        <v>11660</v>
-      </c>
-      <c r="G6" s="1">
-        <v>80</v>
-      </c>
-      <c r="H6" s="1">
-        <v>1117</v>
-      </c>
-      <c r="I6" s="1">
-        <v>1337</v>
+      <c r="B6">
+        <v>15633</v>
+      </c>
+      <c r="C6">
+        <v>100</v>
+      </c>
+      <c r="D6">
+        <v>10810</v>
+      </c>
+      <c r="E6">
+        <v>76</v>
+      </c>
+      <c r="F6">
+        <v>9309</v>
+      </c>
+      <c r="G6">
+        <v>55</v>
+      </c>
+      <c r="H6">
+        <v>2115</v>
+      </c>
+      <c r="I6">
+        <v>2248</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="1">
-        <v>16159</v>
-      </c>
-      <c r="C7" s="1">
-        <v>100</v>
-      </c>
-      <c r="D7" s="1">
-        <v>11534</v>
-      </c>
-      <c r="E7" s="1">
-        <v>83</v>
-      </c>
-      <c r="F7" s="1">
-        <v>9933</v>
-      </c>
-      <c r="G7" s="1">
-        <v>63</v>
-      </c>
-      <c r="H7" s="1">
-        <v>1794</v>
-      </c>
-      <c r="I7" s="1">
-        <v>1981</v>
+      <c r="B7">
+        <v>14682</v>
+      </c>
+      <c r="C7">
+        <v>99</v>
+      </c>
+      <c r="D7">
+        <v>9672</v>
+      </c>
+      <c r="E7">
+        <v>62</v>
+      </c>
+      <c r="F7">
+        <v>8329</v>
+      </c>
+      <c r="G7">
+        <v>41</v>
+      </c>
+      <c r="H7">
+        <v>2724</v>
+      </c>
+      <c r="I7">
+        <v>2696</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="17" x14ac:dyDescent="0.2">

</xml_diff>